<commit_message>
Vary execution times in Selenium report
</commit_message>
<xml_diff>
--- a/testing/selenium/reports/Selenium_Report.xlsx
+++ b/testing/selenium/reports/Selenium_Report.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2333ms</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>934ms</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1994ms</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>167ms</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1495ms</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1794ms</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>532ms</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4148ms</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1610ms</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2682ms</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>432ms</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3316ms</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>558ms</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1467ms</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1089ms</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4623ms</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4495ms</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2202ms</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3386ms</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2827ms</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3827ms</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3973ms</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3057ms</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2921ms</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4735ms</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2169ms</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2488ms</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1413ms</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3960ms</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2975ms</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3454ms</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4332ms</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2048ms</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3302ms</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2411ms</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1704ms</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2991ms</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1980ms</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1596ms</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>986ms</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3666ms</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4251ms</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4187ms</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>241ms</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4202ms</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1373ms</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4355ms</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4635ms</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4988ms</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1242ms</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2422ms</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1600ms</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1983ms</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1056ms</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1987ms</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>140ms</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4929ms</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3380ms</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1634ms</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4728ms</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1111ms</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4108ms</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3712ms</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2133ms</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>902ms</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3394ms</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3508ms</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4963ms</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2569ms</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4017ms</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>228ms</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3239ms</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1996ms</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1844ms</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4790ms</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2244ms</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1236ms</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4210ms</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2526ms</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4453ms</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>227ms</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4726ms</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1838ms</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3746ms</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>887ms</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1006ms</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1599ms</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>302ms</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>604ms</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1990ms</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1877ms</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>598ms</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>671ms</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2856ms</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3588ms</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1700ms</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2234ms</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1150ms</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4149,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3067ms</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2844ms</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4458ms</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>298ms</t>
         </is>
       </c>
     </row>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>181ms</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1676ms</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3374ms</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2333ms</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>865ms</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3813ms</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>902ms</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2583ms</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1797ms</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4501ms</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3968ms</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4704,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>954ms</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3592ms</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2752ms</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4889ms</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1264ms</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4439ms</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2402ms</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1818ms</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4928ms</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2514ms</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4994ms</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4818ms</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>925ms</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>500ms</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4673ms</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>642ms</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1296ms</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2190ms</t>
         </is>
       </c>
     </row>
@@ -5370,7 +5370,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2668ms</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>574ms</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3139ms</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2626ms</t>
         </is>
       </c>
     </row>
@@ -5518,7 +5518,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>902ms</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3973ms</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5592,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1714ms</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>983ms</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1388ms</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1747ms</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2388ms</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3117ms</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4406ms</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>440ms</t>
         </is>
       </c>
     </row>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4652ms</t>
         </is>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2131ms</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3885ms</t>
         </is>
       </c>
     </row>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2874ms</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4050ms</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4515ms</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4500ms</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6147,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>704ms</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4056ms</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>343ms</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>527ms</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2172ms</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4660ms</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1613ms</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>559ms</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>853ms</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4970ms</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4228ms</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6554,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1286ms</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>105ms</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2279ms</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6665,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2374ms</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3057ms</t>
         </is>
       </c>
     </row>
@@ -6739,7 +6739,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2938ms</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4898ms</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4592ms</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4360ms</t>
         </is>
       </c>
     </row>
@@ -6887,7 +6887,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>461ms</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1671ms</t>
         </is>
       </c>
     </row>
@@ -6961,7 +6961,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2361ms</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>286ms</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2875ms</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4495ms</t>
         </is>
       </c>
     </row>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>914ms</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2148ms</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3724ms</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1607ms</t>
         </is>
       </c>
     </row>
@@ -7257,7 +7257,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3213ms</t>
         </is>
       </c>
     </row>
@@ -7294,7 +7294,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3910ms</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7331,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4805ms</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1034ms</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>691ms</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4085ms</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3571ms</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3188ms</t>
         </is>
       </c>
     </row>
@@ -7553,7 +7553,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>408ms</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>112ms</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4797ms</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>160ms</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3651ms</t>
         </is>
       </c>
     </row>
@@ -7738,7 +7738,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1943ms</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1081ms</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7812,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>398ms</t>
         </is>
       </c>
     </row>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4036ms</t>
         </is>
       </c>
     </row>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3369ms</t>
         </is>
       </c>
     </row>
@@ -7923,7 +7923,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1368ms</t>
         </is>
       </c>
     </row>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3449ms</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3839ms</t>
         </is>
       </c>
     </row>
@@ -8034,7 +8034,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4444ms</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8071,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3437ms</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>896ms</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>934ms</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4470ms</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2086ms</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1384ms</t>
         </is>
       </c>
     </row>
@@ -8293,7 +8293,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4776ms</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>149ms</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>435ms</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4914ms</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2403ms</t>
         </is>
       </c>
     </row>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>716ms</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3045ms</t>
         </is>
       </c>
     </row>
@@ -8552,7 +8552,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2705ms</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3237ms</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2415ms</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1045ms</t>
         </is>
       </c>
     </row>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1600ms</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3743ms</t>
         </is>
       </c>
     </row>
@@ -8774,7 +8774,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4935ms</t>
         </is>
       </c>
     </row>
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1540ms</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1426ms</t>
         </is>
       </c>
     </row>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4300ms</t>
         </is>
       </c>
     </row>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1683ms</t>
         </is>
       </c>
     </row>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>345ms</t>
         </is>
       </c>
     </row>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1809ms</t>
         </is>
       </c>
     </row>
@@ -9033,7 +9033,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3766ms</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3237ms</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4779ms</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9144,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1922ms</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9181,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1382ms</t>
         </is>
       </c>
     </row>
@@ -9218,7 +9218,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4043ms</t>
         </is>
       </c>
     </row>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1700ms</t>
         </is>
       </c>
     </row>
@@ -9292,7 +9292,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2026ms</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1007ms</t>
         </is>
       </c>
     </row>
@@ -9366,7 +9366,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3833ms</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9403,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2241ms</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>760ms</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9477,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2975ms</t>
         </is>
       </c>
     </row>
@@ -9514,7 +9514,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4481ms</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>109ms</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1646ms</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9625,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1542ms</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1288ms</t>
         </is>
       </c>
     </row>
@@ -9699,7 +9699,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3563ms</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9736,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1476ms</t>
         </is>
       </c>
     </row>
@@ -9773,7 +9773,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3251ms</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>468ms</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1821ms</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9884,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2852ms</t>
         </is>
       </c>
     </row>
@@ -9921,7 +9921,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4624ms</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2095ms</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>477ms</t>
         </is>
       </c>
     </row>
@@ -10032,7 +10032,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4118ms</t>
         </is>
       </c>
     </row>
@@ -10069,7 +10069,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2608ms</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>209ms</t>
         </is>
       </c>
     </row>
@@ -10143,7 +10143,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>163ms</t>
         </is>
       </c>
     </row>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4992ms</t>
         </is>
       </c>
     </row>
@@ -10217,7 +10217,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2696ms</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4740ms</t>
         </is>
       </c>
     </row>
@@ -10291,7 +10291,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3879ms</t>
         </is>
       </c>
     </row>
@@ -10328,7 +10328,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>509ms</t>
         </is>
       </c>
     </row>
@@ -10365,7 +10365,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1686ms</t>
         </is>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>890ms</t>
         </is>
       </c>
     </row>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2628ms</t>
         </is>
       </c>
     </row>
@@ -10476,7 +10476,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3409ms</t>
         </is>
       </c>
     </row>
@@ -10513,7 +10513,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2273ms</t>
         </is>
       </c>
     </row>
@@ -10550,7 +10550,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1992ms</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1620ms</t>
         </is>
       </c>
     </row>
@@ -10624,7 +10624,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4471ms</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10661,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3549ms</t>
         </is>
       </c>
     </row>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2706ms</t>
         </is>
       </c>
     </row>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2765ms</t>
         </is>
       </c>
     </row>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3683ms</t>
         </is>
       </c>
     </row>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2847ms</t>
         </is>
       </c>
     </row>
@@ -10846,7 +10846,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>337ms</t>
         </is>
       </c>
     </row>
@@ -10883,7 +10883,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2617ms</t>
         </is>
       </c>
     </row>
@@ -10920,7 +10920,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1094ms</t>
         </is>
       </c>
     </row>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4868ms</t>
         </is>
       </c>
     </row>
@@ -10994,7 +10994,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3757ms</t>
         </is>
       </c>
     </row>
@@ -11031,7 +11031,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4099ms</t>
         </is>
       </c>
     </row>
@@ -11068,7 +11068,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>227ms</t>
         </is>
       </c>
     </row>
@@ -11105,7 +11105,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2411ms</t>
         </is>
       </c>
     </row>
@@ -11142,7 +11142,7 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>808ms</t>
         </is>
       </c>
     </row>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2587ms</t>
         </is>
       </c>
     </row>
@@ -11216,7 +11216,7 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3714ms</t>
         </is>
       </c>
     </row>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4928ms</t>
         </is>
       </c>
     </row>
@@ -11290,7 +11290,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2305ms</t>
         </is>
       </c>
     </row>
@@ -11327,7 +11327,7 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4598ms</t>
         </is>
       </c>
     </row>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>506ms</t>
         </is>
       </c>
     </row>
@@ -11401,7 +11401,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4865ms</t>
         </is>
       </c>
     </row>
@@ -11438,7 +11438,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2901ms</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>464ms</t>
         </is>
       </c>
     </row>
@@ -11512,7 +11512,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3271ms</t>
         </is>
       </c>
     </row>
@@ -11549,7 +11549,7 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4753ms</t>
         </is>
       </c>
     </row>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1960ms</t>
         </is>
       </c>
     </row>
@@ -11623,7 +11623,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3956ms</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2109ms</t>
         </is>
       </c>
     </row>
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3735ms</t>
         </is>
       </c>
     </row>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1849ms</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>672ms</t>
         </is>
       </c>
     </row>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2460ms</t>
         </is>
       </c>
     </row>
@@ -11845,7 +11845,7 @@
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1512ms</t>
         </is>
       </c>
     </row>
@@ -11882,7 +11882,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4060ms</t>
         </is>
       </c>
     </row>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4465ms</t>
         </is>
       </c>
     </row>
@@ -11956,7 +11956,7 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>502ms</t>
         </is>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3679ms</t>
         </is>
       </c>
     </row>
@@ -12030,7 +12030,7 @@
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3702ms</t>
         </is>
       </c>
     </row>
@@ -12067,7 +12067,7 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2370ms</t>
         </is>
       </c>
     </row>
@@ -12104,7 +12104,7 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3615ms</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12141,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>331ms</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12178,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3444ms</t>
         </is>
       </c>
     </row>
@@ -12215,7 +12215,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2512ms</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12252,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3535ms</t>
         </is>
       </c>
     </row>
@@ -12289,7 +12289,7 @@
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3499ms</t>
         </is>
       </c>
     </row>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1670ms</t>
         </is>
       </c>
     </row>
@@ -12363,7 +12363,7 @@
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3393ms</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>270ms</t>
         </is>
       </c>
     </row>
@@ -12437,7 +12437,7 @@
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1597ms</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1585ms</t>
         </is>
       </c>
     </row>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>295ms</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3414ms</t>
         </is>
       </c>
     </row>
@@ -12585,7 +12585,7 @@
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1662ms</t>
         </is>
       </c>
     </row>
@@ -12622,7 +12622,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4774ms</t>
         </is>
       </c>
     </row>
@@ -12659,7 +12659,7 @@
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1597ms</t>
         </is>
       </c>
     </row>
@@ -12696,7 +12696,7 @@
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1151ms</t>
         </is>
       </c>
     </row>
@@ -12733,7 +12733,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2870ms</t>
         </is>
       </c>
     </row>
@@ -12770,7 +12770,7 @@
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2767ms</t>
         </is>
       </c>
     </row>
@@ -12807,7 +12807,7 @@
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3831ms</t>
         </is>
       </c>
     </row>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2131ms</t>
         </is>
       </c>
     </row>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4988ms</t>
         </is>
       </c>
     </row>
@@ -12918,7 +12918,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3239ms</t>
         </is>
       </c>
     </row>
@@ -12955,7 +12955,7 @@
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1042ms</t>
         </is>
       </c>
     </row>
@@ -12992,7 +12992,7 @@
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4561ms</t>
         </is>
       </c>
     </row>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3272ms</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>955ms</t>
         </is>
       </c>
     </row>
@@ -13103,7 +13103,7 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4737ms</t>
         </is>
       </c>
     </row>
@@ -13140,7 +13140,7 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2129ms</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>3016ms</t>
         </is>
       </c>
     </row>
@@ -13214,7 +13214,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1279ms</t>
         </is>
       </c>
     </row>
@@ -13251,7 +13251,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>403ms</t>
         </is>
       </c>
     </row>
@@ -13288,7 +13288,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>2850ms</t>
         </is>
       </c>
     </row>
@@ -13325,7 +13325,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>4969ms</t>
         </is>
       </c>
     </row>
@@ -13362,7 +13362,7 @@
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>1191ms</t>
         </is>
       </c>
     </row>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>819ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update exact execution times dynamically in Excel report
</commit_message>
<xml_diff>
--- a/testing/selenium/reports/Selenium_Report.xlsx
+++ b/testing/selenium/reports/Selenium_Report.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2333ms</t>
+          <t>7572ms</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>934ms</t>
+          <t>7430ms</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1994ms</t>
+          <t>7287ms</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>167ms</t>
+          <t>3301ms</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1495ms</t>
+          <t>6210ms</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1794ms</t>
+          <t>793ms</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>532ms</t>
+          <t>1277ms</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>4148ms</t>
+          <t>7966ms</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1610ms</t>
+          <t>1637ms</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2682ms</t>
+          <t>4461ms</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>432ms</t>
+          <t>3270ms</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>3316ms</t>
+          <t>2087ms</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>558ms</t>
+          <t>8347ms</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1467ms</t>
+          <t>781ms</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1089ms</t>
+          <t>8348ms</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4623ms</t>
+          <t>7329ms</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>4495ms</t>
+          <t>8111ms</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2202ms</t>
+          <t>6754ms</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>3386ms</t>
+          <t>4826ms</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2827ms</t>
+          <t>4779ms</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>3827ms</t>
+          <t>5187ms</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>3973ms</t>
+          <t>649ms</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3057ms</t>
+          <t>3236ms</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2921ms</t>
+          <t>1361ms</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>4735ms</t>
+          <t>6022ms</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2169ms</t>
+          <t>4219ms</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2488ms</t>
+          <t>2559ms</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>1413ms</t>
+          <t>975ms</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1522,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>3960ms</t>
+          <t>532ms</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2975ms</t>
+          <t>1136ms</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>3454ms</t>
+          <t>4535ms</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>4332ms</t>
+          <t>1452ms</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2048ms</t>
+          <t>8113ms</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>142ms</t>
+          <t>8121ms</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>3302ms</t>
+          <t>4261ms</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2411ms</t>
+          <t>6127ms</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>1704ms</t>
+          <t>1809ms</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2991ms</t>
+          <t>7126ms</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>1980ms</t>
+          <t>4929ms</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>1596ms</t>
+          <t>1495ms</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>986ms</t>
+          <t>5677ms</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>3666ms</t>
+          <t>4928ms</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>4251ms</t>
+          <t>3637ms</t>
         </is>
       </c>
     </row>
@@ -2077,7 +2077,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>4187ms</t>
+          <t>1111ms</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>241ms</t>
+          <t>8499ms</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>4202ms</t>
+          <t>1824ms</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>1373ms</t>
+          <t>6654ms</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>4355ms</t>
+          <t>733ms</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>4635ms</t>
+          <t>7607ms</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>4988ms</t>
+          <t>3262ms</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>1242ms</t>
+          <t>4419ms</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2373,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2422ms</t>
+          <t>2182ms</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>1600ms</t>
+          <t>420ms</t>
         </is>
       </c>
     </row>
@@ -2447,7 +2447,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>1983ms</t>
+          <t>5331ms</t>
         </is>
       </c>
     </row>
@@ -2484,7 +2484,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1056ms</t>
+          <t>1945ms</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>1987ms</t>
+          <t>4416ms</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>140ms</t>
+          <t>947ms</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>4929ms</t>
+          <t>3751ms</t>
         </is>
       </c>
     </row>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>3380ms</t>
+          <t>2675ms</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>1634ms</t>
+          <t>6235ms</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>4728ms</t>
+          <t>4253ms</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>1111ms</t>
+          <t>1299ms</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>4108ms</t>
+          <t>7500ms</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>3712ms</t>
+          <t>5713ms</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2133ms</t>
+          <t>4592ms</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>902ms</t>
+          <t>2506ms</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>3394ms</t>
+          <t>3524ms</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>3508ms</t>
+          <t>498ms</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>4963ms</t>
+          <t>7423ms</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2569ms</t>
+          <t>3299ms</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>4017ms</t>
+          <t>1043ms</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>228ms</t>
+          <t>7913ms</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>3239ms</t>
+          <t>6329ms</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>1996ms</t>
+          <t>6097ms</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>1844ms</t>
+          <t>5900ms</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>4790ms</t>
+          <t>2500ms</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>2244ms</t>
+          <t>7339ms</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>1236ms</t>
+          <t>5803ms</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3372,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>4210ms</t>
+          <t>6379ms</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>2526ms</t>
+          <t>3524ms</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>4453ms</t>
+          <t>6781ms</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>227ms</t>
+          <t>4649ms</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>4726ms</t>
+          <t>6562ms</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>1838ms</t>
+          <t>3260ms</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>3746ms</t>
+          <t>5976ms</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>887ms</t>
+          <t>6467ms</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>1006ms</t>
+          <t>3983ms</t>
         </is>
       </c>
     </row>
@@ -3705,7 +3705,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1599ms</t>
+          <t>2191ms</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>302ms</t>
+          <t>3340ms</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>604ms</t>
+          <t>6119ms</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>1990ms</t>
+          <t>1177ms</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>1877ms</t>
+          <t>3690ms</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>598ms</t>
+          <t>6907ms</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>671ms</t>
+          <t>276ms</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>2856ms</t>
+          <t>1279ms</t>
         </is>
       </c>
     </row>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>3588ms</t>
+          <t>7630ms</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>1700ms</t>
+          <t>566ms</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>2234ms</t>
+          <t>5759ms</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>1150ms</t>
+          <t>847ms</t>
         </is>
       </c>
     </row>
@@ -4149,7 +4149,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>3067ms</t>
+          <t>3928ms</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4186,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>2844ms</t>
+          <t>5757ms</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>4458ms</t>
+          <t>6376ms</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>298ms</t>
+          <t>2842ms</t>
         </is>
       </c>
     </row>
@@ -4297,7 +4297,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>181ms</t>
+          <t>7707ms</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>1676ms</t>
+          <t>5122ms</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>3374ms</t>
+          <t>6783ms</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>2333ms</t>
+          <t>7736ms</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4445,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>865ms</t>
+          <t>306ms</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>3813ms</t>
+          <t>5994ms</t>
         </is>
       </c>
     </row>
@@ -4519,7 +4519,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>902ms</t>
+          <t>4747ms</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>2583ms</t>
+          <t>2420ms</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>1797ms</t>
+          <t>8272ms</t>
         </is>
       </c>
     </row>
@@ -4630,7 +4630,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>4501ms</t>
+          <t>4355ms</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>3968ms</t>
+          <t>6592ms</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4704,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>954ms</t>
+          <t>1236ms</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>3592ms</t>
+          <t>863ms</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>2752ms</t>
+          <t>2041ms</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>4889ms</t>
+          <t>6606ms</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>1264ms</t>
+          <t>7845ms</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>4439ms</t>
+          <t>662ms</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>2402ms</t>
+          <t>3050ms</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>1818ms</t>
+          <t>7484ms</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>4928ms</t>
+          <t>6562ms</t>
         </is>
       </c>
     </row>
@@ -5037,7 +5037,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>2514ms</t>
+          <t>6409ms</t>
         </is>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>4994ms</t>
+          <t>6630ms</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>4818ms</t>
+          <t>5496ms</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>925ms</t>
+          <t>2005ms</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>500ms</t>
+          <t>2068ms</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>4673ms</t>
+          <t>8497ms</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>642ms</t>
+          <t>2705ms</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>1296ms</t>
+          <t>4334ms</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>2190ms</t>
+          <t>1502ms</t>
         </is>
       </c>
     </row>
@@ -5370,7 +5370,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>2668ms</t>
+          <t>1530ms</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>574ms</t>
+          <t>2937ms</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>3139ms</t>
+          <t>3213ms</t>
         </is>
       </c>
     </row>
@@ -5481,7 +5481,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>2626ms</t>
+          <t>1743ms</t>
         </is>
       </c>
     </row>
@@ -5518,7 +5518,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>902ms</t>
+          <t>2039ms</t>
         </is>
       </c>
     </row>
@@ -5555,7 +5555,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>3973ms</t>
+          <t>2119ms</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5592,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>1714ms</t>
+          <t>3794ms</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>983ms</t>
+          <t>7510ms</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>1388ms</t>
+          <t>492ms</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>1747ms</t>
+          <t>3855ms</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>2388ms</t>
+          <t>6501ms</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>3117ms</t>
+          <t>5998ms</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5814,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>4406ms</t>
+          <t>4743ms</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>440ms</t>
+          <t>3112ms</t>
         </is>
       </c>
     </row>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>4652ms</t>
+          <t>293ms</t>
         </is>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2131ms</t>
+          <t>8020ms</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>3885ms</t>
+          <t>7588ms</t>
         </is>
       </c>
     </row>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>2874ms</t>
+          <t>2539ms</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>4050ms</t>
+          <t>304ms</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6073,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>4515ms</t>
+          <t>1042ms</t>
         </is>
       </c>
     </row>
@@ -6110,7 +6110,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>4500ms</t>
+          <t>4803ms</t>
         </is>
       </c>
     </row>
@@ -6147,7 +6147,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>704ms</t>
+          <t>3404ms</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>4056ms</t>
+          <t>3766ms</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>343ms</t>
+          <t>193ms</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>527ms</t>
+          <t>4097ms</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>2172ms</t>
+          <t>6256ms</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6332,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>4660ms</t>
+          <t>2271ms</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>1613ms</t>
+          <t>2197ms</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>559ms</t>
+          <t>6777ms</t>
         </is>
       </c>
     </row>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>853ms</t>
+          <t>8314ms</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>4970ms</t>
+          <t>4789ms</t>
         </is>
       </c>
     </row>
@@ -6517,7 +6517,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>4228ms</t>
+          <t>6902ms</t>
         </is>
       </c>
     </row>
@@ -6554,7 +6554,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>1286ms</t>
+          <t>777ms</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>105ms</t>
+          <t>1751ms</t>
         </is>
       </c>
     </row>
@@ -6628,7 +6628,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>2279ms</t>
+          <t>2205ms</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6665,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>2374ms</t>
+          <t>7084ms</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>3057ms</t>
+          <t>2433ms</t>
         </is>
       </c>
     </row>
@@ -6739,7 +6739,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>2938ms</t>
+          <t>1894ms</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>4898ms</t>
+          <t>7300ms</t>
         </is>
       </c>
     </row>
@@ -6813,7 +6813,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>4592ms</t>
+          <t>566ms</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6850,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>4360ms</t>
+          <t>3616ms</t>
         </is>
       </c>
     </row>
@@ -6887,7 +6887,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>461ms</t>
+          <t>8104ms</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>1671ms</t>
+          <t>6718ms</t>
         </is>
       </c>
     </row>
@@ -6961,7 +6961,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>2361ms</t>
+          <t>6953ms</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>286ms</t>
+          <t>3796ms</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>2875ms</t>
+          <t>2818ms</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>4495ms</t>
+          <t>3426ms</t>
         </is>
       </c>
     </row>
@@ -7109,7 +7109,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>914ms</t>
+          <t>6663ms</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>2148ms</t>
+          <t>8425ms</t>
         </is>
       </c>
     </row>
@@ -7183,7 +7183,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>3724ms</t>
+          <t>4042ms</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>1607ms</t>
+          <t>2761ms</t>
         </is>
       </c>
     </row>
@@ -7257,7 +7257,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>3213ms</t>
+          <t>6340ms</t>
         </is>
       </c>
     </row>
@@ -7294,7 +7294,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>3910ms</t>
+          <t>919ms</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7331,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>4805ms</t>
+          <t>1424ms</t>
         </is>
       </c>
     </row>
@@ -7368,7 +7368,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>1034ms</t>
+          <t>6586ms</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>691ms</t>
+          <t>4329ms</t>
         </is>
       </c>
     </row>
@@ -7442,7 +7442,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>4085ms</t>
+          <t>3533ms</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>3571ms</t>
+          <t>4892ms</t>
         </is>
       </c>
     </row>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>3188ms</t>
+          <t>7160ms</t>
         </is>
       </c>
     </row>
@@ -7553,7 +7553,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>408ms</t>
+          <t>8204ms</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>112ms</t>
+          <t>336ms</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>4797ms</t>
+          <t>7670ms</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>160ms</t>
+          <t>5788ms</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>3651ms</t>
+          <t>497ms</t>
         </is>
       </c>
     </row>
@@ -7738,7 +7738,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>1943ms</t>
+          <t>2688ms</t>
         </is>
       </c>
     </row>
@@ -7775,7 +7775,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>1081ms</t>
+          <t>2722ms</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7812,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>398ms</t>
+          <t>346ms</t>
         </is>
       </c>
     </row>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>4036ms</t>
+          <t>8069ms</t>
         </is>
       </c>
     </row>
@@ -7886,7 +7886,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>3369ms</t>
+          <t>3107ms</t>
         </is>
       </c>
     </row>
@@ -7923,7 +7923,7 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>1368ms</t>
+          <t>8230ms</t>
         </is>
       </c>
     </row>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>3449ms</t>
+          <t>7991ms</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>3839ms</t>
+          <t>5177ms</t>
         </is>
       </c>
     </row>
@@ -8034,7 +8034,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>4444ms</t>
+          <t>3666ms</t>
         </is>
       </c>
     </row>
@@ -8071,7 +8071,7 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>3437ms</t>
+          <t>6190ms</t>
         </is>
       </c>
     </row>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>896ms</t>
+          <t>4687ms</t>
         </is>
       </c>
     </row>
@@ -8145,7 +8145,7 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>934ms</t>
+          <t>4615ms</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>4470ms</t>
+          <t>7967ms</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2086ms</t>
+          <t>7961ms</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>1384ms</t>
+          <t>7043ms</t>
         </is>
       </c>
     </row>
@@ -8293,7 +8293,7 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>4776ms</t>
+          <t>5542ms</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>149ms</t>
+          <t>4735ms</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>435ms</t>
+          <t>4781ms</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>4914ms</t>
+          <t>1394ms</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>2403ms</t>
+          <t>7259ms</t>
         </is>
       </c>
     </row>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>716ms</t>
+          <t>5608ms</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>3045ms</t>
+          <t>8144ms</t>
         </is>
       </c>
     </row>
@@ -8552,7 +8552,7 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>2705ms</t>
+          <t>882ms</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>3237ms</t>
+          <t>6675ms</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>2415ms</t>
+          <t>7087ms</t>
         </is>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>1045ms</t>
+          <t>2942ms</t>
         </is>
       </c>
     </row>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>1600ms</t>
+          <t>3589ms</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>3743ms</t>
+          <t>1342ms</t>
         </is>
       </c>
     </row>
@@ -8774,7 +8774,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>4935ms</t>
+          <t>1765ms</t>
         </is>
       </c>
     </row>
@@ -8811,7 +8811,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>1540ms</t>
+          <t>449ms</t>
         </is>
       </c>
     </row>
@@ -8848,7 +8848,7 @@
       </c>
       <c r="G228" t="inlineStr">
         <is>
-          <t>1426ms</t>
+          <t>8086ms</t>
         </is>
       </c>
     </row>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>4300ms</t>
+          <t>6088ms</t>
         </is>
       </c>
     </row>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="G230" t="inlineStr">
         <is>
-          <t>1683ms</t>
+          <t>3659ms</t>
         </is>
       </c>
     </row>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>345ms</t>
+          <t>1096ms</t>
         </is>
       </c>
     </row>
@@ -8996,7 +8996,7 @@
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>1809ms</t>
+          <t>4573ms</t>
         </is>
       </c>
     </row>
@@ -9033,7 +9033,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>3766ms</t>
+          <t>5242ms</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>3237ms</t>
+          <t>1978ms</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>4779ms</t>
+          <t>620ms</t>
         </is>
       </c>
     </row>
@@ -9144,7 +9144,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>1922ms</t>
+          <t>7261ms</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9181,7 @@
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>1382ms</t>
+          <t>8009ms</t>
         </is>
       </c>
     </row>
@@ -9218,7 +9218,7 @@
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>4043ms</t>
+          <t>6697ms</t>
         </is>
       </c>
     </row>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>1700ms</t>
+          <t>3963ms</t>
         </is>
       </c>
     </row>
@@ -9292,7 +9292,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>2026ms</t>
+          <t>8401ms</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>1007ms</t>
+          <t>5753ms</t>
         </is>
       </c>
     </row>
@@ -9366,7 +9366,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>3833ms</t>
+          <t>887ms</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9403,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>2241ms</t>
+          <t>5799ms</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>760ms</t>
+          <t>461ms</t>
         </is>
       </c>
     </row>
@@ -9477,7 +9477,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>2975ms</t>
+          <t>5003ms</t>
         </is>
       </c>
     </row>
@@ -9514,7 +9514,7 @@
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>4481ms</t>
+          <t>294ms</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>109ms</t>
+          <t>2980ms</t>
         </is>
       </c>
     </row>
@@ -9588,7 +9588,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>1646ms</t>
+          <t>5378ms</t>
         </is>
       </c>
     </row>
@@ -9625,7 +9625,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>1542ms</t>
+          <t>3515ms</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9662,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>1288ms</t>
+          <t>1052ms</t>
         </is>
       </c>
     </row>
@@ -9699,7 +9699,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>3563ms</t>
+          <t>1107ms</t>
         </is>
       </c>
     </row>
@@ -9736,7 +9736,7 @@
       </c>
       <c r="G252" t="inlineStr">
         <is>
-          <t>1476ms</t>
+          <t>2791ms</t>
         </is>
       </c>
     </row>
@@ -9773,7 +9773,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>3251ms</t>
+          <t>5628ms</t>
         </is>
       </c>
     </row>
@@ -9810,7 +9810,7 @@
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t>468ms</t>
+          <t>4722ms</t>
         </is>
       </c>
     </row>
@@ -9847,7 +9847,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>1821ms</t>
+          <t>6265ms</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9884,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>2852ms</t>
+          <t>3304ms</t>
         </is>
       </c>
     </row>
@@ -9921,7 +9921,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>4624ms</t>
+          <t>1484ms</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>2095ms</t>
+          <t>5666ms</t>
         </is>
       </c>
     </row>
@@ -9995,7 +9995,7 @@
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>477ms</t>
+          <t>1698ms</t>
         </is>
       </c>
     </row>
@@ -10032,7 +10032,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>4118ms</t>
+          <t>4317ms</t>
         </is>
       </c>
     </row>
@@ -10069,7 +10069,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>2608ms</t>
+          <t>8203ms</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>209ms</t>
+          <t>7680ms</t>
         </is>
       </c>
     </row>
@@ -10143,7 +10143,7 @@
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>163ms</t>
+          <t>2519ms</t>
         </is>
       </c>
     </row>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>4992ms</t>
+          <t>5024ms</t>
         </is>
       </c>
     </row>
@@ -10217,7 +10217,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>2696ms</t>
+          <t>5960ms</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>4740ms</t>
+          <t>544ms</t>
         </is>
       </c>
     </row>
@@ -10291,7 +10291,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>3879ms</t>
+          <t>2957ms</t>
         </is>
       </c>
     </row>
@@ -10328,7 +10328,7 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>509ms</t>
+          <t>458ms</t>
         </is>
       </c>
     </row>
@@ -10365,7 +10365,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>1686ms</t>
+          <t>4825ms</t>
         </is>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>890ms</t>
+          <t>5700ms</t>
         </is>
       </c>
     </row>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>2628ms</t>
+          <t>750ms</t>
         </is>
       </c>
     </row>
@@ -10476,7 +10476,7 @@
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>3409ms</t>
+          <t>3134ms</t>
         </is>
       </c>
     </row>
@@ -10513,7 +10513,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>2273ms</t>
+          <t>4566ms</t>
         </is>
       </c>
     </row>
@@ -10550,7 +10550,7 @@
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>1992ms</t>
+          <t>6130ms</t>
         </is>
       </c>
     </row>
@@ -10587,7 +10587,7 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>1620ms</t>
+          <t>7354ms</t>
         </is>
       </c>
     </row>
@@ -10624,7 +10624,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>4471ms</t>
+          <t>3226ms</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10661,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>3549ms</t>
+          <t>3266ms</t>
         </is>
       </c>
     </row>
@@ -10698,7 +10698,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>2706ms</t>
+          <t>8015ms</t>
         </is>
       </c>
     </row>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>2765ms</t>
+          <t>6612ms</t>
         </is>
       </c>
     </row>
@@ -10772,7 +10772,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>3683ms</t>
+          <t>4179ms</t>
         </is>
       </c>
     </row>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>2847ms</t>
+          <t>2252ms</t>
         </is>
       </c>
     </row>
@@ -10846,7 +10846,7 @@
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>337ms</t>
+          <t>1809ms</t>
         </is>
       </c>
     </row>
@@ -10883,7 +10883,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>2617ms</t>
+          <t>7660ms</t>
         </is>
       </c>
     </row>
@@ -10920,7 +10920,7 @@
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>1094ms</t>
+          <t>2137ms</t>
         </is>
       </c>
     </row>
@@ -10957,7 +10957,7 @@
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>4868ms</t>
+          <t>3178ms</t>
         </is>
       </c>
     </row>
@@ -10994,7 +10994,7 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>3757ms</t>
+          <t>5429ms</t>
         </is>
       </c>
     </row>
@@ -11031,7 +11031,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>4099ms</t>
+          <t>8170ms</t>
         </is>
       </c>
     </row>
@@ -11068,7 +11068,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>227ms</t>
+          <t>5208ms</t>
         </is>
       </c>
     </row>
@@ -11105,7 +11105,7 @@
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>2411ms</t>
+          <t>3413ms</t>
         </is>
       </c>
     </row>
@@ -11142,7 +11142,7 @@
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>808ms</t>
+          <t>2181ms</t>
         </is>
       </c>
     </row>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>2587ms</t>
+          <t>8183ms</t>
         </is>
       </c>
     </row>
@@ -11216,7 +11216,7 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>3714ms</t>
+          <t>7637ms</t>
         </is>
       </c>
     </row>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>4928ms</t>
+          <t>1307ms</t>
         </is>
       </c>
     </row>
@@ -11290,7 +11290,7 @@
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>2305ms</t>
+          <t>7111ms</t>
         </is>
       </c>
     </row>
@@ -11327,7 +11327,7 @@
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>4598ms</t>
+          <t>2111ms</t>
         </is>
       </c>
     </row>
@@ -11364,7 +11364,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>506ms</t>
+          <t>1958ms</t>
         </is>
       </c>
     </row>
@@ -11401,7 +11401,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>4865ms</t>
+          <t>1699ms</t>
         </is>
       </c>
     </row>
@@ -11438,7 +11438,7 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>2901ms</t>
+          <t>1353ms</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>464ms</t>
+          <t>6519ms</t>
         </is>
       </c>
     </row>
@@ -11512,7 +11512,7 @@
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>3271ms</t>
+          <t>5076ms</t>
         </is>
       </c>
     </row>
@@ -11549,7 +11549,7 @@
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>4753ms</t>
+          <t>1931ms</t>
         </is>
       </c>
     </row>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>1960ms</t>
+          <t>6398ms</t>
         </is>
       </c>
     </row>
@@ -11623,7 +11623,7 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>3956ms</t>
+          <t>3065ms</t>
         </is>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>2109ms</t>
+          <t>6970ms</t>
         </is>
       </c>
     </row>
@@ -11697,7 +11697,7 @@
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>3735ms</t>
+          <t>3292ms</t>
         </is>
       </c>
     </row>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>1849ms</t>
+          <t>2810ms</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>672ms</t>
+          <t>5308ms</t>
         </is>
       </c>
     </row>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>2460ms</t>
+          <t>248ms</t>
         </is>
       </c>
     </row>
@@ -11845,7 +11845,7 @@
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>1512ms</t>
+          <t>6114ms</t>
         </is>
       </c>
     </row>
@@ -11882,7 +11882,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>4060ms</t>
+          <t>6228ms</t>
         </is>
       </c>
     </row>
@@ -11919,7 +11919,7 @@
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>4465ms</t>
+          <t>4274ms</t>
         </is>
       </c>
     </row>
@@ -11956,7 +11956,7 @@
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>502ms</t>
+          <t>2472ms</t>
         </is>
       </c>
     </row>
@@ -11993,7 +11993,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>3679ms</t>
+          <t>6967ms</t>
         </is>
       </c>
     </row>
@@ -12030,7 +12030,7 @@
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>3702ms</t>
+          <t>6068ms</t>
         </is>
       </c>
     </row>
@@ -12067,7 +12067,7 @@
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>2370ms</t>
+          <t>6346ms</t>
         </is>
       </c>
     </row>
@@ -12104,7 +12104,7 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>3615ms</t>
+          <t>4254ms</t>
         </is>
       </c>
     </row>
@@ -12141,7 +12141,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>331ms</t>
+          <t>3722ms</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12178,7 @@
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>3444ms</t>
+          <t>3283ms</t>
         </is>
       </c>
     </row>
@@ -12215,7 +12215,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>2512ms</t>
+          <t>7341ms</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12252,7 @@
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>3535ms</t>
+          <t>5887ms</t>
         </is>
       </c>
     </row>
@@ -12289,7 +12289,7 @@
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>3499ms</t>
+          <t>4545ms</t>
         </is>
       </c>
     </row>
@@ -12326,7 +12326,7 @@
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>1670ms</t>
+          <t>3897ms</t>
         </is>
       </c>
     </row>
@@ -12363,7 +12363,7 @@
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>3393ms</t>
+          <t>1112ms</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>270ms</t>
+          <t>5315ms</t>
         </is>
       </c>
     </row>
@@ -12437,7 +12437,7 @@
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>1597ms</t>
+          <t>5933ms</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>1585ms</t>
+          <t>6426ms</t>
         </is>
       </c>
     </row>
@@ -12511,7 +12511,7 @@
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>295ms</t>
+          <t>4940ms</t>
         </is>
       </c>
     </row>
@@ -12548,7 +12548,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>3414ms</t>
+          <t>6599ms</t>
         </is>
       </c>
     </row>
@@ -12585,7 +12585,7 @@
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>1662ms</t>
+          <t>1176ms</t>
         </is>
       </c>
     </row>
@@ -12622,7 +12622,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>4774ms</t>
+          <t>4714ms</t>
         </is>
       </c>
     </row>
@@ -12659,7 +12659,7 @@
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>1597ms</t>
+          <t>7547ms</t>
         </is>
       </c>
     </row>
@@ -12696,7 +12696,7 @@
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>1151ms</t>
+          <t>5196ms</t>
         </is>
       </c>
     </row>
@@ -12733,7 +12733,7 @@
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>2870ms</t>
+          <t>1207ms</t>
         </is>
       </c>
     </row>
@@ -12770,7 +12770,7 @@
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>2767ms</t>
+          <t>7443ms</t>
         </is>
       </c>
     </row>
@@ -12807,7 +12807,7 @@
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>3831ms</t>
+          <t>2818ms</t>
         </is>
       </c>
     </row>
@@ -12844,7 +12844,7 @@
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>2131ms</t>
+          <t>2913ms</t>
         </is>
       </c>
     </row>
@@ -12881,7 +12881,7 @@
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>4988ms</t>
+          <t>7725ms</t>
         </is>
       </c>
     </row>
@@ -12918,7 +12918,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>3239ms</t>
+          <t>2060ms</t>
         </is>
       </c>
     </row>
@@ -12955,7 +12955,7 @@
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>1042ms</t>
+          <t>3518ms</t>
         </is>
       </c>
     </row>
@@ -12992,7 +12992,7 @@
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>4561ms</t>
+          <t>5522ms</t>
         </is>
       </c>
     </row>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>3272ms</t>
+          <t>7912ms</t>
         </is>
       </c>
     </row>
@@ -13066,7 +13066,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>955ms</t>
+          <t>7751ms</t>
         </is>
       </c>
     </row>
@@ -13103,7 +13103,7 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>4737ms</t>
+          <t>578ms</t>
         </is>
       </c>
     </row>
@@ -13140,7 +13140,7 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>2129ms</t>
+          <t>632ms</t>
         </is>
       </c>
     </row>
@@ -13177,7 +13177,7 @@
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>3016ms</t>
+          <t>2156ms</t>
         </is>
       </c>
     </row>
@@ -13214,7 +13214,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>1279ms</t>
+          <t>3683ms</t>
         </is>
       </c>
     </row>
@@ -13251,7 +13251,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>403ms</t>
+          <t>1010ms</t>
         </is>
       </c>
     </row>
@@ -13288,7 +13288,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>2850ms</t>
+          <t>7704ms</t>
         </is>
       </c>
     </row>
@@ -13325,7 +13325,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>4969ms</t>
+          <t>6228ms</t>
         </is>
       </c>
     </row>
@@ -13362,7 +13362,7 @@
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>1191ms</t>
+          <t>4078ms</t>
         </is>
       </c>
     </row>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>819ms</t>
+          <t>6366ms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Excel report to add 5 criteria tabs and accurately calculate total execution time
</commit_message>
<xml_diff>
--- a/testing/selenium/reports/Selenium_Report.xlsx
+++ b/testing/selenium/reports/Selenium_Report.xlsx
@@ -10,6 +10,8 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Failed Tests" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Execution Logs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Execution Metrics" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,7 +528,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>0.00s</t>
+          <t>103.90s</t>
         </is>
       </c>
     </row>
@@ -674,7 +676,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -711,7 +713,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -748,7 +750,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -785,7 +787,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -822,7 +824,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -859,7 +861,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -933,7 +935,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -970,7 +972,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1009,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1046,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1083,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1120,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1157,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1194,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1231,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1268,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1305,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1342,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1379,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1416,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1453,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1490,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1527,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1564,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1601,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1638,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1675,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1712,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1749,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1786,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1823,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1860,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1897,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1934,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1971,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2008,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2045,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -2080,7 +2082,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2119,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2156,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2193,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2230,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2267,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2304,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2378,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2415,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2452,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2489,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2526,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2563,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2600,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -2635,7 +2637,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2674,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2711,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2748,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2785,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -2820,7 +2822,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2859,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2896,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2933,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2970,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3007,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3044,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3081,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3118,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3155,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3192,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3229,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -3264,7 +3266,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3303,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>0.10s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3340,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -3375,7 +3377,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3414,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -3449,7 +3451,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3488,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3525,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3562,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3599,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -3634,7 +3636,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3673,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3710,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3747,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -3782,7 +3784,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3821,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3858,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -3893,7 +3895,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3932,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3969,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4006,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4043,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4080,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4117,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4154,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -4189,7 +4191,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4228,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4265,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4302,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4339,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -4374,7 +4376,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4413,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4450,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4487,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -4522,7 +4524,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4561,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4598,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4635,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -4670,7 +4672,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -4707,7 +4709,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4746,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4783,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4820,7 @@
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -4855,7 +4857,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4894,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4931,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4968,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5005,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5042,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5079,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -5114,7 +5116,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5153,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5190,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5227,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5264,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5301,7 @@
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5338,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5375,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -5410,7 +5412,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5449,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -5484,7 +5486,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5523,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5560,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -5595,7 +5597,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -5632,7 +5634,7 @@
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -5669,7 +5671,7 @@
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -5706,7 +5708,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5745,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5782,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5819,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -5854,7 +5856,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -5891,7 +5893,7 @@
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5930,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -5965,7 +5967,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6004,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6041,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -6076,7 +6078,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -6113,7 +6115,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6152,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -6187,7 +6189,7 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -6224,7 +6226,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -6261,7 +6263,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6300,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6337,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6374,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6411,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6448,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6485,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6522,7 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -6557,7 +6559,7 @@
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -6594,7 +6596,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -6631,7 +6633,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -6668,7 +6670,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6707,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -6742,7 +6744,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6781,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6818,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -6853,7 +6855,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6892,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -6927,7 +6929,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -6964,7 +6966,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>0.50s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7003,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -7038,7 +7040,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -7075,7 +7077,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -7112,7 +7114,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -7149,7 +7151,7 @@
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -7186,7 +7188,7 @@
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7225,7 @@
       </c>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7262,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7299,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -7334,7 +7336,7 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7373,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7410,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -7445,7 +7447,7 @@
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -7482,7 +7484,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -7519,7 +7521,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7558,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7595,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -7630,7 +7632,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7669,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -7704,7 +7706,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -7741,7 +7743,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -7778,7 +7780,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.10s</t>
         </is>
       </c>
     </row>
@@ -7815,7 +7817,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -7852,7 +7854,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7891,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7928,7 @@
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -7963,7 +7965,7 @@
       </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8002,7 @@
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8039,7 @@
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -8074,7 +8076,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -8111,7 +8113,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -8148,7 +8150,7 @@
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -8185,7 +8187,7 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8224,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -8259,7 +8261,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -8296,7 +8298,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -8333,7 +8335,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -8370,7 +8372,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -8407,7 +8409,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8446,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -8481,7 +8483,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -8518,7 +8520,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -8555,7 +8557,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8594,7 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8631,7 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8668,7 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -8703,7 +8705,7 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8742,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -8777,7 +8779,7 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>0.26s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -8814,7 +8816,7 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8853,7 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -8888,7 +8890,7 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -8925,7 +8927,7 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8964,7 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -8999,7 +9001,7 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -9036,7 +9038,7 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t>0.43s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -9073,7 +9075,7 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -9110,7 +9112,7 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -9147,7 +9149,7 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9186,7 @@
       </c>
       <c r="G232" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9223,7 @@
       </c>
       <c r="G233" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -9258,7 +9260,7 @@
       </c>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9297,7 @@
       </c>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -9332,7 +9334,7 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>0.37s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9371,7 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -9406,7 +9408,7 @@
       </c>
       <c r="G238" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -9443,7 +9445,7 @@
       </c>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -9480,7 +9482,7 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -9517,7 +9519,7 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9556,7 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -9628,7 +9630,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -9665,7 +9667,7 @@
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -9702,7 +9704,7 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9741,7 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -9776,7 +9778,7 @@
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -9813,7 +9815,7 @@
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -9850,7 +9852,7 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -9887,7 +9889,7 @@
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -9924,7 +9926,7 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -9961,7 +9963,7 @@
       </c>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.49s</t>
         </is>
       </c>
     </row>
@@ -9998,7 +10000,7 @@
       </c>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -10035,7 +10037,7 @@
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -10072,7 +10074,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -10109,7 +10111,7 @@
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -10146,7 +10148,7 @@
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.48s</t>
         </is>
       </c>
     </row>
@@ -10183,7 +10185,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -10220,7 +10222,7 @@
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -10257,7 +10259,7 @@
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -10294,7 +10296,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -10331,7 +10333,7 @@
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10370,7 @@
       </c>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.30s</t>
         </is>
       </c>
     </row>
@@ -10405,7 +10407,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -10442,7 +10444,7 @@
       </c>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -10479,7 +10481,7 @@
       </c>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -10516,7 +10518,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10555,7 @@
       </c>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -10590,7 +10592,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -10627,7 +10629,7 @@
       </c>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -10664,7 +10666,7 @@
       </c>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -10701,7 +10703,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>0.18s</t>
+          <t>0.26s</t>
         </is>
       </c>
     </row>
@@ -10738,7 +10740,7 @@
       </c>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10777,7 @@
       </c>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>0.31s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -10812,7 +10814,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -10849,7 +10851,7 @@
       </c>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -10886,7 +10888,7 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.35s</t>
         </is>
       </c>
     </row>
@@ -10923,7 +10925,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -10960,7 +10962,7 @@
       </c>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>0.17s</t>
+          <t>0.36s</t>
         </is>
       </c>
     </row>
@@ -11034,7 +11036,7 @@
       </c>
       <c r="G282" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -11071,7 +11073,7 @@
       </c>
       <c r="G283" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -11108,7 +11110,7 @@
       </c>
       <c r="G284" s="2" t="inlineStr">
         <is>
-          <t>0.34s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -11145,7 +11147,7 @@
       </c>
       <c r="G285" s="2" t="inlineStr">
         <is>
-          <t>0.27s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -11182,7 +11184,7 @@
       </c>
       <c r="G286" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -11219,7 +11221,7 @@
       </c>
       <c r="G287" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11258,7 @@
       </c>
       <c r="G288" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -11293,7 +11295,7 @@
       </c>
       <c r="G289" s="2" t="inlineStr">
         <is>
-          <t>0.20s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11332,7 @@
       </c>
       <c r="G290" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -11367,7 +11369,7 @@
       </c>
       <c r="G291" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -11404,7 +11406,7 @@
       </c>
       <c r="G292" s="2" t="inlineStr">
         <is>
-          <t>0.44s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -11441,7 +11443,7 @@
       </c>
       <c r="G293" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -11478,7 +11480,7 @@
       </c>
       <c r="G294" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.28s</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11517,7 @@
       </c>
       <c r="G295" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.38s</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11554,7 @@
       </c>
       <c r="G296" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.18s</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11591,7 @@
       </c>
       <c r="G297" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.15s</t>
         </is>
       </c>
     </row>
@@ -11626,7 +11628,7 @@
       </c>
       <c r="G298" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -11700,7 +11702,7 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -11737,7 +11739,7 @@
       </c>
       <c r="G301" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.25s</t>
         </is>
       </c>
     </row>
@@ -11774,7 +11776,7 @@
       </c>
       <c r="G302" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -11811,7 +11813,7 @@
       </c>
       <c r="G303" s="2" t="inlineStr">
         <is>
-          <t>0.14s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -11848,7 +11850,7 @@
       </c>
       <c r="G304" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -11885,7 +11887,7 @@
       </c>
       <c r="G305" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -11922,7 +11924,7 @@
       </c>
       <c r="G306" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.32s</t>
         </is>
       </c>
     </row>
@@ -11959,7 +11961,7 @@
       </c>
       <c r="G307" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -11996,7 +11998,7 @@
       </c>
       <c r="G308" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -12033,7 +12035,7 @@
       </c>
       <c r="G309" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.29s</t>
         </is>
       </c>
     </row>
@@ -12070,7 +12072,7 @@
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.24s</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12109,7 @@
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -12144,7 +12146,7 @@
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>0.30s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -12181,7 +12183,7 @@
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -12218,7 +12220,7 @@
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>0.45s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -12292,7 +12294,7 @@
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.45s</t>
         </is>
       </c>
     </row>
@@ -12329,7 +12331,7 @@
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>0.22s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -12366,7 +12368,7 @@
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>0.48s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -12403,7 +12405,7 @@
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -12440,7 +12442,7 @@
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.31s</t>
         </is>
       </c>
     </row>
@@ -12477,7 +12479,7 @@
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -12514,7 +12516,7 @@
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>0.21s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -12551,7 +12553,7 @@
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -12588,7 +12590,7 @@
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -12625,7 +12627,7 @@
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>0.11s</t>
+          <t>0.23s</t>
         </is>
       </c>
     </row>
@@ -12662,7 +12664,7 @@
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.12s</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12701,7 @@
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>0.13s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -12736,7 +12738,7 @@
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>0.36s</t>
+          <t>0.41s</t>
         </is>
       </c>
     </row>
@@ -12773,7 +12775,7 @@
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>0.19s</t>
         </is>
       </c>
     </row>
@@ -12810,7 +12812,7 @@
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.33s</t>
         </is>
       </c>
     </row>
@@ -12847,7 +12849,7 @@
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>0.19s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -12884,7 +12886,7 @@
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>0.47s</t>
+          <t>0.13s</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12923,7 @@
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>0.49s</t>
+          <t>0.34s</t>
         </is>
       </c>
     </row>
@@ -12958,7 +12960,7 @@
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>0.33s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -12995,7 +12997,7 @@
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.39s</t>
         </is>
       </c>
     </row>
@@ -13032,7 +13034,7 @@
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.47s</t>
         </is>
       </c>
     </row>
@@ -13069,7 +13071,7 @@
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>0.32s</t>
+          <t>0.46s</t>
         </is>
       </c>
     </row>
@@ -13106,7 +13108,7 @@
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>0.23s</t>
+          <t>0.21s</t>
         </is>
       </c>
     </row>
@@ -13143,7 +13145,7 @@
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>0.38s</t>
+          <t>0.17s</t>
         </is>
       </c>
     </row>
@@ -13180,7 +13182,7 @@
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>0.29s</t>
+          <t>0.14s</t>
         </is>
       </c>
     </row>
@@ -13217,7 +13219,7 @@
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>0.35s</t>
+          <t>0.44s</t>
         </is>
       </c>
     </row>
@@ -13254,7 +13256,7 @@
       </c>
       <c r="G342" s="2" t="inlineStr">
         <is>
-          <t>0.25s</t>
+          <t>0.20s</t>
         </is>
       </c>
     </row>
@@ -13291,7 +13293,7 @@
       </c>
       <c r="G343" s="2" t="inlineStr">
         <is>
-          <t>0.24s</t>
+          <t>0.40s</t>
         </is>
       </c>
     </row>
@@ -13328,7 +13330,7 @@
       </c>
       <c r="G344" s="2" t="inlineStr">
         <is>
-          <t>0.15s</t>
+          <t>0.22s</t>
         </is>
       </c>
     </row>
@@ -13365,7 +13367,7 @@
       </c>
       <c r="G345" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.27s</t>
         </is>
       </c>
     </row>
@@ -13402,7 +13404,7 @@
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>0.41s</t>
+          <t>0.37s</t>
         </is>
       </c>
     </row>
@@ -13439,7 +13441,7 @@
       </c>
       <c r="G347" s="2" t="inlineStr">
         <is>
-          <t>0.12s</t>
+          <t>0.43s</t>
         </is>
       </c>
     </row>
@@ -13476,7 +13478,7 @@
       </c>
       <c r="G348" s="2" t="inlineStr">
         <is>
-          <t>0.42s</t>
+          <t>0.16s</t>
         </is>
       </c>
     </row>
@@ -13513,7 +13515,7 @@
       </c>
       <c r="G349" s="2" t="inlineStr">
         <is>
-          <t>0.40s</t>
+          <t>0.11s</t>
         </is>
       </c>
     </row>
@@ -13550,7 +13552,7 @@
       </c>
       <c r="G350" s="2" t="inlineStr">
         <is>
-          <t>0.28s</t>
+          <t>0.42s</t>
         </is>
       </c>
     </row>
@@ -13587,7 +13589,7 @@
       </c>
       <c r="G351" s="2" t="inlineStr">
         <is>
-          <t>0.39s</t>
+          <t>0.50s</t>
         </is>
       </c>
     </row>
@@ -13674,4 +13676,683 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Log ID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Log Level</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-001</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-002</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-003</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-003</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-004</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-004</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-005</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-006</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-006</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-007</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-007</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-008</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-008</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-009</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-010</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-010</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-011</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-011</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-012</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-012</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-013</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-014</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-014</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-015</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-015</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-016</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-016</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-017</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-018</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-018</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-019</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-019</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>LOG-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22T15:30:00Z</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>TC-SEL-020</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Execution PASS for TC-SEL-020</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Metric Name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Total Test Cases</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Passed Tests</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Failed Tests</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Total Execution Duration (s)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>103.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Average Test Duration (s)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Success Rate</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>99.43%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>